<commit_message>
PCB V2, CAD V3 & Code
</commit_message>
<xml_diff>
--- a/Mechanical/Buying List.xlsx
+++ b/Mechanical/Buying List.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\angel\Desktop\Proyectos\FOC_BLDC\Mechanical\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DF5D17A-30EF-4F7D-8806-47D19973AA62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{729BE44D-F2ED-4F66-AFE8-7EE9039F2437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Components" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="45">
   <si>
     <t>Component</t>
   </si>
@@ -1192,10 +1192,10 @@
         <v>0</v>
       </c>
       <c r="F3" s="23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G3" s="25" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H3" s="14">
         <f>Table1[[#This Row],[Unit Price]]*Table1[[#This Row],[Quantity]]+Table1[[#This Row],[Shipping Costs]]</f>
@@ -1283,7 +1283,7 @@
         <v>25</v>
       </c>
       <c r="G6" s="25" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H6" s="14">
         <v>64.11</v>
@@ -1308,7 +1308,7 @@
         <v>25</v>
       </c>
       <c r="G7" s="25" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H7" s="14">
         <f>Table1[[#This Row],[Unit Price]]*Table1[[#This Row],[Quantity]]+Table1[[#This Row],[Shipping Costs]]</f>
@@ -1336,7 +1336,7 @@
         <v>25</v>
       </c>
       <c r="G8" s="25" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H8" s="14">
         <f>Table1[[#This Row],[Unit Price]]*Table1[[#This Row],[Quantity]]+Table1[[#This Row],[Shipping Costs]]</f>
@@ -1365,8 +1365,8 @@
       <c r="F9" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="G9" s="25">
-        <v>1</v>
+      <c r="G9" s="25" t="s">
+        <v>25</v>
       </c>
       <c r="H9" s="14">
         <f>Table1[[#This Row],[Unit Price]]*Table1[[#This Row],[Quantity]]+Table1[[#This Row],[Shipping Costs]]</f>

</xml_diff>